<commit_message>
41.1: Added new categories, hobbies, deeds, etc.
</commit_message>
<xml_diff>
--- a/SourceFiles/DeedInfo-4-The War.xlsx
+++ b/SourceFiles/DeedInfo-4-The War.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119C66CE-8D19-41BB-B5D4-6E0EED6E726B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586BBED8-0A20-4F8C-8C51-A99CCC0D8C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="465" windowWidth="24435" windowHeight="14865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="204">
   <si>
     <t>Save Index</t>
   </si>
@@ -624,6 +624,33 @@
   </si>
   <si>
     <t>Defeat 500 Weavers in the Ettenmoors</t>
+  </si>
+  <si>
+    <t>Title: Protector of Life</t>
+  </si>
+  <si>
+    <t>Title: Steward of the Ettenmoors</t>
+  </si>
+  <si>
+    <t>Title: Servant of Shadow</t>
+  </si>
+  <si>
+    <t>Title: Preserver of Order</t>
+  </si>
+  <si>
+    <t>- Monster Player Reward Season 1 -</t>
+  </si>
+  <si>
+    <t>Title: Angmar's Enforcer</t>
+  </si>
+  <si>
+    <t>Title: Abomination</t>
+  </si>
+  <si>
+    <t>Title: Exemplar</t>
+  </si>
+  <si>
+    <t>Title: Scourge of the Ettenmoors</t>
   </si>
 </sst>
 </file>
@@ -673,10 +700,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -809,6 +837,7 @@
       <sheetName val="The War of Three Peaks"/>
       <sheetName val="The Mountain-hold"/>
       <sheetName val="Return to Carn Dûm"/>
+      <sheetName val="Corsairs of Umbar"/>
       <sheetName val="&lt;template&gt;"/>
     </sheetNames>
     <sheetDataSet>
@@ -1609,6 +1638,7 @@
       <sheetData sheetId="18"/>
       <sheetData sheetId="19"/>
       <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -8245,6 +8275,7 @@
     <col min="18" max="18" width="12.140625" customWidth="1"/>
     <col min="19" max="19" width="18" customWidth="1"/>
     <col min="25" max="25" width="14" customWidth="1"/>
+    <col min="27" max="27" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" x14ac:dyDescent="0.25">
@@ -8415,7 +8446,7 @@
       </c>
       <c r="S2" s="1" t="str">
         <f>CONCATENATE(U2,V2,Y2,AA2,AC2,AE2,AG2,AI2,AK2,AL2,AM2,AN2,AO2,AP2,AQ2,AR2,AS2)</f>
-        <v xml:space="preserve">  [1] = {["ID"] = 1879071835; ["SAVE_INDEX"] = 1; ["TYPE"] = 4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of Tol Ascarnen"; }; ["LORE"] = { ["EN"] = "Defeat the enemy Chieftains controlling the fortress of Tol Ascarnen!"; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of Tol Ascarnen"; }; };</v>
+        <v xml:space="preserve">  [1] = {["ID"] = 1879071835; ["SAVE_INDEX"] = 1; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of Tol Ascarnen"; }; ["LORE"] = { ["EN"] = "Defeat the enemy Chieftains controlling the fortress of Tol Ascarnen!"; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of Tol Ascarnen"; }; };</v>
       </c>
       <c r="T2">
         <f>ROW()-1</f>
@@ -8446,8 +8477,8 @@
         <v>4</v>
       </c>
       <c r="AA2" t="str">
-        <f>CONCATENATE("[""TYPE""] = ",REPT(" ",1-LEN(Z2)),Z2,"; ")</f>
-        <v xml:space="preserve">["TYPE"] = 4; </v>
+        <f>CONCATENATE("[""TYPE""] = ",REPT(" ",2-LEN(Z2)),Z2,"; ")</f>
+        <v xml:space="preserve">["TYPE"] =  4; </v>
       </c>
       <c r="AB2" t="str">
         <f>IF(NOT(ISBLANK(E2)),VLOOKUP(E2,[1]Type!D$2:E$6,2,FALSE),"")</f>
@@ -8553,10 +8584,10 @@
       </c>
       <c r="S3" s="1" t="str">
         <f t="shared" ref="S3:S5" si="2">CONCATENATE(U3,V3,Y3,AA3,AC3,AE3,AG3,AI3,AK3,AL3,AM3,AN3,AO3,AP3,AQ3,AR3,AS3)</f>
-        <v xml:space="preserve">  [2] = {["ID"] = 1879071836; ["SAVE_INDEX"] = 2; ["TYPE"] = 4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of Dargazag"; }; ["LORE"] = { ["EN"] = "The Enemy's forces in the field are led by a number of Chieftans. Defeating them all will weaken the morale of their forces, and deny them leadership."; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of Dargazag"; }; };</v>
+        <v xml:space="preserve">  [2] = {["ID"] = 1879071836; ["SAVE_INDEX"] = 2; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of Dargazag"; }; ["LORE"] = { ["EN"] = "The Enemy's forces in the field are led by a number of Chieftans. Defeating them all will weaken the morale of their forces, and deny them leadership."; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of Dargazag"; }; };</v>
       </c>
       <c r="T3">
-        <f t="shared" ref="T3:T5" si="3">ROW()-1</f>
+        <f t="shared" ref="T3:T19" si="3">ROW()-1</f>
         <v>2</v>
       </c>
       <c r="U3" t="str">
@@ -8584,8 +8615,8 @@
         <v>4</v>
       </c>
       <c r="AA3" t="str">
-        <f t="shared" ref="AA3:AA5" si="9">CONCATENATE("[""TYPE""] = ",REPT(" ",1-LEN(Z3)),Z3,"; ")</f>
-        <v xml:space="preserve">["TYPE"] = 4; </v>
+        <f t="shared" ref="AA3:AA19" si="9">CONCATENATE("[""TYPE""] = ",REPT(" ",2-LEN(Z3)),Z3,"; ")</f>
+        <v xml:space="preserve">["TYPE"] =  4; </v>
       </c>
       <c r="AB3" t="str">
         <f>IF(NOT(ISBLANK(E3)),VLOOKUP(E3,[1]Type!D$2:E$6,2,FALSE),"")</f>
@@ -8640,7 +8671,7 @@
         <v/>
       </c>
       <c r="AO3" t="str">
-        <f t="shared" ref="AO3:AO5" si="21">CONCATENATE("[""NAME""] = { [""EN""] = """,C3,"""; }; ")</f>
+        <f t="shared" ref="AO3:AO6" si="21">CONCATENATE("[""NAME""] = { [""EN""] = """,C3,"""; }; ")</f>
         <v xml:space="preserve">["NAME"] = { ["EN"] = "Conquest of Dargazag"; }; </v>
       </c>
       <c r="AP3" t="str">
@@ -8656,7 +8687,7 @@
         <v xml:space="preserve">["TITLE"] = { ["EN"] = "Conqueror of Dargazag"; }; </v>
       </c>
       <c r="AS3" t="str">
-        <f t="shared" ref="AS3:AS5" si="25">CONCATENATE("};")</f>
+        <f t="shared" ref="AS3:AS19" si="25">CONCATENATE("};")</f>
         <v>};</v>
       </c>
     </row>
@@ -8691,7 +8722,7 @@
       </c>
       <c r="S4" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [3] = {["ID"] = 1879071837; ["SAVE_INDEX"] = 3; ["TYPE"] = 4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of the Towers"; }; ["LORE"] = { ["EN"] = "Two strong towers oversee the defences of the Ettenmoors, defeat the enemy chieftains inhabiting these towers!"; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of the Towers"; }; };</v>
+        <v xml:space="preserve">  [3] = {["ID"] = 1879071837; ["SAVE_INDEX"] = 3; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "50"; ["NAME"] = { ["EN"] = "Conquest of the Towers"; }; ["LORE"] = { ["EN"] = "Two strong towers oversee the defences of the Ettenmoors, defeat the enemy chieftains inhabiting these towers!"; }; ["SUMMARY"] = { ["EN"] = "Defeat 4 chieftains"; }; ["TITLE"] = { ["EN"] = "Conqueror of the Towers"; }; };</v>
       </c>
       <c r="T4">
         <f t="shared" si="3"/>
@@ -8723,7 +8754,7 @@
       </c>
       <c r="AA4" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve">["TYPE"] = 4; </v>
+        <v xml:space="preserve">["TYPE"] =  4; </v>
       </c>
       <c r="AB4" t="str">
         <f>IF(NOT(ISBLANK(E4)),VLOOKUP(E4,[1]Type!D$2:E$6,2,FALSE),"")</f>
@@ -8829,7 +8860,7 @@
       </c>
       <c r="S5" s="1" t="str">
         <f t="shared" si="2"/>
-        <v xml:space="preserve">  [4] = {["ID"] = 1879071838; ["SAVE_INDEX"] = 4; ["TYPE"] = 4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "45"; ["NAME"] = { ["EN"] = "Tyrants of the Enemy"; }; ["LORE"] = { ["EN"] = "Find and defeat the Tyrants of the forces of the Enemy in the Ettenmoors, ensuring the victory of the armies of the West."; }; ["SUMMARY"] = { ["EN"] = "Defeat 6 tyrants"; }; ["TITLE"] = { ["EN"] = "Conqueror of the Ettenmoors"; }; };</v>
+        <v xml:space="preserve">  [4] = {["ID"] = 1879071838; ["SAVE_INDEX"] = 4; ["TYPE"] =  4; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["MIN_LVL"] = "45"; ["NAME"] = { ["EN"] = "Tyrants of the Enemy"; }; ["LORE"] = { ["EN"] = "Find and defeat the Tyrants of the forces of the Enemy in the Ettenmoors, ensuring the victory of the armies of the West."; }; ["SUMMARY"] = { ["EN"] = "Defeat 6 tyrants"; }; ["TITLE"] = { ["EN"] = "Conqueror of the Ettenmoors"; }; };</v>
       </c>
       <c r="T5">
         <f t="shared" si="3"/>
@@ -8861,7 +8892,7 @@
       </c>
       <c r="AA5" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve">["TYPE"] = 4; </v>
+        <v xml:space="preserve">["TYPE"] =  4; </v>
       </c>
       <c r="AB5" t="str">
         <f>IF(NOT(ISBLANK(E5)),VLOOKUP(E5,[1]Type!D$2:E$6,2,FALSE),"")</f>
@@ -8937,148 +8968,1762 @@
       </c>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="S6" s="1"/>
-      <c r="Y6" s="1"/>
+      <c r="C6" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="P6">
+        <v>308</v>
+      </c>
+      <c r="R6" t="str">
+        <f t="shared" ref="R6:R19" si="26">CONCATENATE(U6,W6,X6,AS6," -- ",C6)</f>
+        <v xml:space="preserve">  [5] = {["CAT_ID"] = 308; }; -- - Monster Player Reward Season 1 -</v>
+      </c>
+      <c r="S6" s="1" t="str">
+        <f t="shared" ref="S6:S19" si="27">CONCATENATE(U6,V6,Y6,AA6,AC6,AE6,AG6,AI6,AK6,AL6,AM6,AN6,AO6,AP6,AQ6,AR6,AS6)</f>
+        <v xml:space="preserve">  [5] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Monster Player Reward Season 1 -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="U6" t="str">
+        <f t="shared" ref="U6:U19" si="28">CONCATENATE(REPT(" ",3-LEN(T6)),"[",T6,"] = {")</f>
+        <v xml:space="preserve">  [5] = {</v>
+      </c>
+      <c r="V6" t="str">
+        <f t="shared" ref="V6:V19" si="29">IF(LEN(A6)&gt;0,CONCATENATE("[""ID""] = ",A6,"; "),"                     ")</f>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W6" t="str">
+        <f t="shared" ref="W6:W19" si="30">IF(LEN(A6)&gt;0,CONCATENATE("[""ID""] = ",A6,"; "),"")</f>
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <f t="shared" ref="X6:X19" si="31">IF(LEN(P6)&gt;0,CONCATENATE("[""CAT_ID""] = ",P6,"; "),"")</f>
+        <v xml:space="preserve">["CAT_ID"] = 308; </v>
+      </c>
+      <c r="Y6" s="1" t="str">
+        <f t="shared" ref="Y6:Y19" si="32">IF(LEN(B6)&gt;0,CONCATENATE("[""SAVE_INDEX""] = ",REPT(" ",1-LEN(B6)),B6,"; "),REPT(" ",20))</f>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z6">
+        <f>VLOOKUP(D6,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>14</v>
+      </c>
+      <c r="AA6" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] = 14; </v>
+      </c>
+      <c r="AB6" t="str">
+        <f>IF(NOT(ISBLANK(E6)),VLOOKUP(E6,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC6" t="str">
+        <f t="shared" ref="AC6:AC19" si="33">IF(NOT(ISBLANK(E6)),CONCATENATE("[""NA""] = ",AB6,"; "),"")</f>
+        <v/>
+      </c>
+      <c r="AD6" t="str">
+        <f t="shared" ref="AD6:AD19" si="34">TEXT(F6,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AE6" t="str">
+        <f t="shared" ref="AE6:AE19" si="35">CONCATENATE("[""VXP""] = ",REPT(" ",1-LEN(AD6)),TEXT(AD6,"0"),"; ")</f>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF6" t="str">
+        <f t="shared" ref="AF6:AF19" si="36">TEXT(H6,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AG6" t="str">
+        <f t="shared" ref="AG6:AG19" si="37">CONCATENATE("[""LP""] = ",REPT(" ",1-LEN(AF6)),TEXT(AF6,"0"),"; ")</f>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH6" t="str">
+        <f t="shared" ref="AH6:AH19" si="38">TEXT(I6,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AI6" t="str">
+        <f t="shared" ref="AI6:AI19" si="39">CONCATENATE("[""REP""] = ",REPT(" ",1-LEN(AH6)),TEXT(AH6,"0"),"; ")</f>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ6">
+        <f>IF(NOT(ISBLANK(J6)),VLOOKUP(J6,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK6" t="str">
+        <f t="shared" ref="AK6:AK19" si="40">CONCATENATE("[""FACTION""] = ",TEXT(AJ6,"0"),"; ")</f>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL6" t="str">
+        <f t="shared" ref="AL6:AL19" si="41">CONCATENATE("[""TIER""] = ",TEXT(M6,"0"),"; ")</f>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM6" t="str">
+        <f t="shared" ref="AM6:AM19" si="42">IF(LEN(N6)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",2-LEN(N6)),"""",N6,"""; "),"")</f>
+        <v/>
+      </c>
+      <c r="AN6" t="str">
+        <f t="shared" ref="AN6:AN19" si="43">IF(LEN(O6)&gt;0,CONCATENATE("[""MIN_LVL""] = ",REPT(" ",3-LEN(O6)),"""",O6,"""; "),"")</f>
+        <v/>
+      </c>
+      <c r="AO6" t="str">
+        <f t="shared" ref="AO6:AO19" si="44">CONCATENATE("[""NAME""] = { [""EN""] = """,C6,"""; }; ")</f>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Monster Player Reward Season 1 -"; }; </v>
+      </c>
+      <c r="AP6" t="str">
+        <f t="shared" ref="AP6:AP19" si="45">CONCATENATE("[""LORE""] = { [""EN""] = """,L6,"""; }; ")</f>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ6" t="str">
+        <f t="shared" ref="AQ6:AQ19" si="46">CONCATENATE("[""SUMMARY""] = { [""EN""] = """,K6,"""; }; ")</f>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR6" t="str">
+        <f t="shared" ref="AR6:AR19" si="47">IF(LEN(G6)&gt;0,CONCATENATE("[""TITLE""] = { [""EN""] = """,G6,"""; }; "),"")</f>
+        <v/>
+      </c>
+      <c r="AS6" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="7" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1879490385</v>
+      </c>
+      <c r="C7" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" t="s">
+        <v>154</v>
+      </c>
       <c r="N7" s="2"/>
-      <c r="S7" s="1"/>
-      <c r="Y7" s="1"/>
+      <c r="R7" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  [6] = {["ID"] = 1879490385; }; -- Title: Protector of Life</v>
+      </c>
+      <c r="S7" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  [6] = {["ID"] = 1879490385;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Protector of Life"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="U7" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  [6] = {</v>
+      </c>
+      <c r="V7" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490385; </v>
+      </c>
+      <c r="W7" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490385; </v>
+      </c>
+      <c r="X7" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y7" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z7">
+        <f>VLOOKUP(D7,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA7" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB7" t="str">
+        <f>IF(NOT(ISBLANK(E7)),VLOOKUP(E7,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC7" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD7" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE7" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF7" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG7" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH7" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI7" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ7">
+        <f>IF(NOT(ISBLANK(J7)),VLOOKUP(J7,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK7" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL7" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM7" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN7" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO7" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Protector of Life"; }; </v>
+      </c>
+      <c r="AP7" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ7" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR7" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS7" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="8" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D8" s="2"/>
+      <c r="A8">
+        <v>1879490388</v>
+      </c>
+      <c r="C8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D8" t="s">
+        <v>154</v>
+      </c>
       <c r="N8" s="2"/>
-      <c r="S8" s="1"/>
-      <c r="Y8" s="1"/>
+      <c r="R8" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879490388; }; -- Title: Steward of the Ettenmoors</v>
+      </c>
+      <c r="S8" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  [7] = {["ID"] = 1879490388;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Steward of the Ettenmoors"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="U8" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  [7] = {</v>
+      </c>
+      <c r="V8" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490388; </v>
+      </c>
+      <c r="W8" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490388; </v>
+      </c>
+      <c r="X8" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y8" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z8">
+        <f>VLOOKUP(D8,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA8" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB8" t="str">
+        <f>IF(NOT(ISBLANK(E8)),VLOOKUP(E8,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC8" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD8" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE8" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF8" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG8" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH8" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI8" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ8">
+        <f>IF(NOT(ISBLANK(J8)),VLOOKUP(J8,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK8" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL8" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM8" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN8" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO8" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Steward of the Ettenmoors"; }; </v>
+      </c>
+      <c r="AP8" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ8" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR8" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS8" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="9" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D9" s="2"/>
+      <c r="A9">
+        <v>1879490389</v>
+      </c>
+      <c r="C9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" t="s">
+        <v>154</v>
+      </c>
       <c r="N9" s="2"/>
-      <c r="S9" s="1"/>
-      <c r="Y9" s="1"/>
+      <c r="R9" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  [8] = {["ID"] = 1879490389; }; -- Title: Servant of Shadow</v>
+      </c>
+      <c r="S9" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  [8] = {["ID"] = 1879490389;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Servant of Shadow"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="U9" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  [8] = {</v>
+      </c>
+      <c r="V9" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490389; </v>
+      </c>
+      <c r="W9" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490389; </v>
+      </c>
+      <c r="X9" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y9" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z9">
+        <f>VLOOKUP(D9,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA9" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB9" t="str">
+        <f>IF(NOT(ISBLANK(E9)),VLOOKUP(E9,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC9" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD9" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE9" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF9" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG9" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH9" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI9" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ9">
+        <f>IF(NOT(ISBLANK(J9)),VLOOKUP(J9,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK9" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL9" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM9" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN9" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO9" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Servant of Shadow"; }; </v>
+      </c>
+      <c r="AP9" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ9" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR9" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS9" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="10" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D10" s="2"/>
+      <c r="A10">
+        <v>1879490390</v>
+      </c>
+      <c r="C10" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" t="s">
+        <v>154</v>
+      </c>
       <c r="N10" s="2"/>
-      <c r="S10" s="1"/>
-      <c r="Y10" s="1"/>
+      <c r="R10" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve">  [9] = {["ID"] = 1879490390; }; -- Title: Preserver of Order</v>
+      </c>
+      <c r="S10" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve">  [9] = {["ID"] = 1879490390;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Preserver of Order"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="U10" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve">  [9] = {</v>
+      </c>
+      <c r="V10" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490390; </v>
+      </c>
+      <c r="W10" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490390; </v>
+      </c>
+      <c r="X10" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y10" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z10">
+        <f>VLOOKUP(D10,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA10" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB10" t="str">
+        <f>IF(NOT(ISBLANK(E10)),VLOOKUP(E10,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC10" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD10" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE10" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF10" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG10" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH10" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI10" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ10">
+        <f>IF(NOT(ISBLANK(J10)),VLOOKUP(J10,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK10" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL10" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM10" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN10" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO10" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Preserver of Order"; }; </v>
+      </c>
+      <c r="AP10" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ10" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR10" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS10" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="11" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D11" s="2"/>
+      <c r="A11">
+        <v>1879490391</v>
+      </c>
+      <c r="C11" t="s">
+        <v>200</v>
+      </c>
+      <c r="D11" t="s">
+        <v>154</v>
+      </c>
       <c r="N11" s="2"/>
-      <c r="S11" s="1"/>
-      <c r="Y11" s="1"/>
+      <c r="R11" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [10] = {["ID"] = 1879490391; }; -- Title: Angmar's Enforcer</v>
+      </c>
+      <c r="S11" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve"> [10] = {["ID"] = 1879490391;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Angmar's Enforcer"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="U11" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [10] = {</v>
+      </c>
+      <c r="V11" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490391; </v>
+      </c>
+      <c r="W11" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490391; </v>
+      </c>
+      <c r="X11" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y11" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z11">
+        <f>VLOOKUP(D11,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA11" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB11" t="str">
+        <f>IF(NOT(ISBLANK(E11)),VLOOKUP(E11,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC11" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD11" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE11" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF11" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG11" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH11" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI11" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ11">
+        <f>IF(NOT(ISBLANK(J11)),VLOOKUP(J11,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK11" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL11" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM11" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN11" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO11" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Angmar's Enforcer"; }; </v>
+      </c>
+      <c r="AP11" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ11" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR11" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS11" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="12" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D12" s="2"/>
+      <c r="A12">
+        <v>1879490392</v>
+      </c>
+      <c r="C12" t="s">
+        <v>201</v>
+      </c>
+      <c r="D12" t="s">
+        <v>154</v>
+      </c>
       <c r="N12" s="2"/>
-      <c r="S12" s="1"/>
-      <c r="Y12" s="1"/>
+      <c r="R12" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [11] = {["ID"] = 1879490392; }; -- Title: Abomination</v>
+      </c>
+      <c r="S12" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve"> [11] = {["ID"] = 1879490392;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Abomination"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="U12" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [11] = {</v>
+      </c>
+      <c r="V12" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490392; </v>
+      </c>
+      <c r="W12" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490392; </v>
+      </c>
+      <c r="X12" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y12" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z12">
+        <f>VLOOKUP(D12,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA12" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB12" t="str">
+        <f>IF(NOT(ISBLANK(E12)),VLOOKUP(E12,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC12" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD12" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE12" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF12" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG12" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH12" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI12" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ12">
+        <f>IF(NOT(ISBLANK(J12)),VLOOKUP(J12,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK12" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL12" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM12" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN12" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO12" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Abomination"; }; </v>
+      </c>
+      <c r="AP12" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ12" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR12" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS12" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="13" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D13" s="2"/>
+      <c r="A13">
+        <v>1879490393</v>
+      </c>
+      <c r="C13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" t="s">
+        <v>154</v>
+      </c>
       <c r="N13" s="2"/>
-      <c r="S13" s="1"/>
-      <c r="Y13" s="1"/>
+      <c r="R13" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [12] = {["ID"] = 1879490393; }; -- Title: Exemplar</v>
+      </c>
+      <c r="S13" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve"> [12] = {["ID"] = 1879490393;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Exemplar"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="U13" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [12] = {</v>
+      </c>
+      <c r="V13" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490393; </v>
+      </c>
+      <c r="W13" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490393; </v>
+      </c>
+      <c r="X13" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y13" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z13">
+        <f>VLOOKUP(D13,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA13" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB13" t="str">
+        <f>IF(NOT(ISBLANK(E13)),VLOOKUP(E13,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC13" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD13" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE13" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF13" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG13" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH13" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI13" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ13">
+        <f>IF(NOT(ISBLANK(J13)),VLOOKUP(J13,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK13" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL13" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM13" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN13" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO13" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Exemplar"; }; </v>
+      </c>
+      <c r="AP13" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ13" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR13" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS13" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="14" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D14" s="2"/>
+      <c r="A14">
+        <v>1879490394</v>
+      </c>
+      <c r="C14" t="s">
+        <v>203</v>
+      </c>
+      <c r="D14" t="s">
+        <v>154</v>
+      </c>
       <c r="N14" s="2"/>
-      <c r="S14" s="1"/>
-      <c r="Y14" s="1"/>
+      <c r="R14" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [13] = {["ID"] = 1879490394; }; -- Title: Scourge of the Ettenmoors</v>
+      </c>
+      <c r="S14" s="1" t="str">
+        <f t="shared" si="27"/>
+        <v xml:space="preserve"> [13] = {["ID"] = 1879490394;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Title: Scourge of the Ettenmoors"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="U14" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [13] = {</v>
+      </c>
+      <c r="V14" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">["ID"] = 1879490394; </v>
+      </c>
+      <c r="W14" t="str">
+        <f t="shared" si="30"/>
+        <v xml:space="preserve">["ID"] = 1879490394; </v>
+      </c>
+      <c r="X14" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y14" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z14">
+        <f>VLOOKUP(D14,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="AA14" t="str">
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
+      </c>
+      <c r="AB14" t="str">
+        <f>IF(NOT(ISBLANK(E14)),VLOOKUP(E14,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC14" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD14" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE14" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF14" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG14" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH14" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI14" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ14">
+        <f>IF(NOT(ISBLANK(J14)),VLOOKUP(J14,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK14" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL14" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM14" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN14" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO14" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Title: Scourge of the Ettenmoors"; }; </v>
+      </c>
+      <c r="AP14" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ14" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR14" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS14" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.25">
       <c r="D15" s="2"/>
       <c r="N15" s="2"/>
-      <c r="S15" s="1"/>
-      <c r="Y15" s="1"/>
+      <c r="R15" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [14] = {}; -- </v>
+      </c>
+      <c r="S15" s="1" t="e">
+        <f t="shared" si="27"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="U15" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [14] = {</v>
+      </c>
+      <c r="V15" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W15" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y15" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z15" t="e">
+        <f>VLOOKUP(D15,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AA15" t="e">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="AB15" t="str">
+        <f>IF(NOT(ISBLANK(E15)),VLOOKUP(E15,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC15" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD15" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE15" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF15" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG15" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH15" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI15" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ15">
+        <f>IF(NOT(ISBLANK(J15)),VLOOKUP(J15,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK15" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL15" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM15" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN15" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO15" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AP15" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ15" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR15" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS15" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
     </row>
     <row r="16" spans="1:45" x14ac:dyDescent="0.25">
       <c r="D16" s="2"/>
       <c r="N16" s="2"/>
-      <c r="S16" s="1"/>
-      <c r="Y16" s="1"/>
-    </row>
-    <row r="17" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="R16" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [15] = {}; -- </v>
+      </c>
+      <c r="S16" s="1" t="e">
+        <f t="shared" si="27"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="U16" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [15] = {</v>
+      </c>
+      <c r="V16" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W16" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y16" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z16" t="e">
+        <f>VLOOKUP(D16,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AA16" t="e">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="AB16" t="str">
+        <f>IF(NOT(ISBLANK(E16)),VLOOKUP(E16,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC16" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD16" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE16" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF16" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG16" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH16" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI16" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ16">
+        <f>IF(NOT(ISBLANK(J16)),VLOOKUP(J16,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK16" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL16" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM16" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN16" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO16" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AP16" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ16" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR16" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS16" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="17" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D17" s="2"/>
       <c r="N17" s="2"/>
-      <c r="S17" s="1"/>
-      <c r="Y17" s="1"/>
-    </row>
-    <row r="18" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="R17" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [16] = {}; -- </v>
+      </c>
+      <c r="S17" s="1" t="e">
+        <f t="shared" si="27"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T17">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="U17" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [16] = {</v>
+      </c>
+      <c r="V17" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W17" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y17" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z17" t="e">
+        <f>VLOOKUP(D17,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AA17" t="e">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="AB17" t="str">
+        <f>IF(NOT(ISBLANK(E17)),VLOOKUP(E17,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC17" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD17" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE17" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF17" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG17" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH17" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI17" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ17">
+        <f>IF(NOT(ISBLANK(J17)),VLOOKUP(J17,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK17" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL17" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM17" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN17" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO17" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AP17" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ17" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR17" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS17" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="18" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D18" s="2"/>
       <c r="N18" s="2"/>
-      <c r="S18" s="1"/>
-      <c r="Y18" s="1"/>
-    </row>
-    <row r="19" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="R18" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [17] = {}; -- </v>
+      </c>
+      <c r="S18" s="1" t="e">
+        <f t="shared" si="27"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="3"/>
+        <v>17</v>
+      </c>
+      <c r="U18" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [17] = {</v>
+      </c>
+      <c r="V18" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W18" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y18" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z18" t="e">
+        <f>VLOOKUP(D18,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AA18" t="e">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="AB18" t="str">
+        <f>IF(NOT(ISBLANK(E18)),VLOOKUP(E18,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC18" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD18" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE18" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF18" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG18" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH18" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI18" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ18">
+        <f>IF(NOT(ISBLANK(J18)),VLOOKUP(J18,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK18" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL18" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM18" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN18" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO18" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AP18" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ18" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR18" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS18" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="19" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D19" s="2"/>
       <c r="N19" s="2"/>
-      <c r="S19" s="1"/>
-      <c r="Y19" s="1"/>
-    </row>
-    <row r="20" spans="4:25" x14ac:dyDescent="0.25">
+      <c r="R19" t="str">
+        <f t="shared" si="26"/>
+        <v xml:space="preserve"> [18] = {}; -- </v>
+      </c>
+      <c r="S19" s="1" t="e">
+        <f t="shared" si="27"/>
+        <v>#N/A</v>
+      </c>
+      <c r="T19">
+        <f t="shared" si="3"/>
+        <v>18</v>
+      </c>
+      <c r="U19" t="str">
+        <f t="shared" si="28"/>
+        <v xml:space="preserve"> [18] = {</v>
+      </c>
+      <c r="V19" t="str">
+        <f t="shared" si="29"/>
+        <v xml:space="preserve">                     </v>
+      </c>
+      <c r="W19" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+      <c r="Y19" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v xml:space="preserve">                    </v>
+      </c>
+      <c r="Z19" t="e">
+        <f>VLOOKUP(D19,[1]Type!A$2:B$18,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="AA19" t="e">
+        <f t="shared" si="9"/>
+        <v>#N/A</v>
+      </c>
+      <c r="AB19" t="str">
+        <f>IF(NOT(ISBLANK(E19)),VLOOKUP(E19,[1]Type!D$2:E$6,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="AC19" t="str">
+        <f t="shared" si="33"/>
+        <v/>
+      </c>
+      <c r="AD19" t="str">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="AE19" t="str">
+        <f t="shared" si="35"/>
+        <v xml:space="preserve">["VXP"] = 0; </v>
+      </c>
+      <c r="AF19" t="str">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="AG19" t="str">
+        <f t="shared" si="37"/>
+        <v xml:space="preserve">["LP"] = 0; </v>
+      </c>
+      <c r="AH19" t="str">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="AI19" t="str">
+        <f t="shared" si="39"/>
+        <v xml:space="preserve">["REP"] = 0; </v>
+      </c>
+      <c r="AJ19">
+        <f>IF(NOT(ISBLANK(J19)),VLOOKUP(J19,[1]Faction!A$2:B$77,2,FALSE),1)</f>
+        <v>1</v>
+      </c>
+      <c r="AK19" t="str">
+        <f t="shared" si="40"/>
+        <v xml:space="preserve">["FACTION"] = 1; </v>
+      </c>
+      <c r="AL19" t="str">
+        <f t="shared" si="41"/>
+        <v xml:space="preserve">["TIER"] = 0; </v>
+      </c>
+      <c r="AM19" t="str">
+        <f t="shared" si="42"/>
+        <v/>
+      </c>
+      <c r="AN19" t="str">
+        <f t="shared" si="43"/>
+        <v/>
+      </c>
+      <c r="AO19" t="str">
+        <f t="shared" si="44"/>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AP19" t="str">
+        <f t="shared" si="45"/>
+        <v xml:space="preserve">["LORE"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AQ19" t="str">
+        <f t="shared" si="46"/>
+        <v xml:space="preserve">["SUMMARY"] = { ["EN"] = ""; }; </v>
+      </c>
+      <c r="AR19" t="str">
+        <f t="shared" si="47"/>
+        <v/>
+      </c>
+      <c r="AS19" t="str">
+        <f t="shared" si="25"/>
+        <v>};</v>
+      </c>
+    </row>
+    <row r="20" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D20" s="2"/>
       <c r="N20" s="2"/>
       <c r="S20" s="1"/>
       <c r="Y20" s="1"/>
     </row>
-    <row r="21" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D21" s="2"/>
       <c r="N21" s="2"/>
       <c r="S21" s="1"/>
       <c r="Y21" s="1"/>
     </row>
-    <row r="22" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D22" s="2"/>
       <c r="N22" s="2"/>
       <c r="S22" s="1"/>
       <c r="Y22" s="1"/>
     </row>
-    <row r="23" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D23" s="2"/>
       <c r="N23" s="2"/>
       <c r="S23" s="1"/>
       <c r="Y23" s="1"/>
     </row>
-    <row r="24" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D24" s="2"/>
       <c r="N24" s="2"/>
       <c r="S24" s="1"/>
       <c r="Y24" s="1"/>
     </row>
-    <row r="25" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:45" x14ac:dyDescent="0.25">
       <c r="D25" s="2"/>
       <c r="N25" s="2"/>
       <c r="S25" s="1"/>
       <c r="Y25" s="1"/>
     </row>
-    <row r="26" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:45" x14ac:dyDescent="0.25">
       <c r="N26" s="2"/>
       <c r="S26" s="1"/>
       <c r="Y26" s="1"/>
     </row>
-    <row r="27" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:45" x14ac:dyDescent="0.25">
       <c r="S27" s="1"/>
       <c r="Y27" s="1"/>
     </row>
-    <row r="28" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:45" x14ac:dyDescent="0.25">
       <c r="S28" s="1"/>
       <c r="Y28" s="1"/>
     </row>
-    <row r="29" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:45" x14ac:dyDescent="0.25">
       <c r="S29" s="1"/>
       <c r="Y29" s="1"/>
     </row>
-    <row r="30" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:45" x14ac:dyDescent="0.25">
       <c r="S30" s="1"/>
       <c r="Y30" s="1"/>
     </row>
-    <row r="31" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="31" spans="4:45" x14ac:dyDescent="0.25">
       <c r="S31" s="1"/>
       <c r="Y31" s="1"/>
     </row>
-    <row r="32" spans="4:25" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:45" x14ac:dyDescent="0.25">
       <c r="S32" s="1"/>
       <c r="Y32" s="1"/>
     </row>

</xml_diff>